<commit_message>
refactor: transform_contas_recebidas_fechamento.py trata os valores do vl_baixa que contém P no corpo.
</commit_message>
<xml_diff>
--- a/stages/extract/reference/auxiliar_contas_recebidas_socios.xlsx
+++ b/stages/extract/reference/auxiliar_contas_recebidas_socios.xlsx
@@ -12,6 +12,9 @@
     <sheet name="condicoes_pagamento" sheetId="2" state="visible" r:id="rId4"/>
     <sheet name="tipos_cliente" sheetId="3" state="visible" r:id="rId5"/>
   </sheets>
+  <definedNames>
+    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">centros_custo!$A$1:$I$16</definedName>
+  </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
@@ -458,6 +461,47 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
+  <dxfs count="5">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF1F4E79"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFDCE6F1"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF000000"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFFFFF"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <colors>
     <indexedColors>
       <rgbColor rgb="FF000000"/>
@@ -519,6 +563,10 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1135,6 +1183,7 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:I16"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -1142,6 +1191,7 @@
     <oddHeader/>
     <oddFooter/>
   </headerFooter>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
refactor: eliminar redundancias nos extracts
</commit_message>
<xml_diff>
--- a/stages/extract/reference/auxiliar_contas_recebidas_socios.xlsx
+++ b/stages/extract/reference/auxiliar_contas_recebidas_socios.xlsx
@@ -66,6 +66,9 @@
     <t xml:space="preserve">GRAND PALAZZO</t>
   </si>
   <si>
+    <t xml:space="preserve">não</t>
+  </si>
+  <si>
     <t xml:space="preserve">nao</t>
   </si>
   <si>
@@ -91,9 +94,6 @@
   </si>
   <si>
     <t xml:space="preserve">RESIDENCIAL RESERVA DOS PASSAROS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">não</t>
   </si>
   <si>
     <t xml:space="preserve">RESIDENCIAL GRAND RESERVA MODULO I</t>
@@ -834,11 +834,11 @@
       <c r="F3" s="6" t="n">
         <v>45292</v>
       </c>
-      <c r="G3" s="3" t="s">
-        <v>11</v>
+      <c r="G3" s="1" t="s">
+        <v>13</v>
       </c>
       <c r="I3" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -846,13 +846,13 @@
         <v>120</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C4" s="1" t="n">
         <v>1</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E4" s="5" t="n">
         <v>0.1001</v>
@@ -860,8 +860,8 @@
       <c r="F4" s="9" t="n">
         <v>44927</v>
       </c>
-      <c r="G4" s="3" t="s">
-        <v>11</v>
+      <c r="G4" s="1" t="s">
+        <v>13</v>
       </c>
       <c r="I4" s="1" t="s">
         <v>11</v>
@@ -872,7 +872,7 @@
         <v>138</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C5" s="1" t="n">
         <v>1</v>
@@ -886,8 +886,8 @@
       <c r="F5" s="6" t="n">
         <v>45658</v>
       </c>
-      <c r="G5" s="3" t="s">
-        <v>11</v>
+      <c r="G5" s="1" t="s">
+        <v>13</v>
       </c>
       <c r="I5" s="1" t="s">
         <v>11</v>
@@ -895,13 +895,13 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C6" s="1" t="n">
         <v>9</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E6" s="10" t="n">
         <v>0.1288</v>
@@ -909,25 +909,25 @@
       <c r="F6" s="9" t="n">
         <v>46023</v>
       </c>
-      <c r="G6" s="3" t="s">
-        <v>11</v>
+      <c r="G6" s="1" t="s">
+        <v>13</v>
       </c>
       <c r="H6" s="9" t="n">
         <v>44197</v>
       </c>
       <c r="I6" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C7" s="1" t="n">
         <v>10</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E7" s="10" t="n">
         <v>0.1288</v>
@@ -935,19 +935,19 @@
       <c r="F7" s="9" t="n">
         <v>46023</v>
       </c>
-      <c r="G7" s="3" t="s">
-        <v>11</v>
+      <c r="G7" s="1" t="s">
+        <v>13</v>
       </c>
       <c r="H7" s="9" t="n">
         <v>43831</v>
       </c>
       <c r="I7" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="7" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C8" s="1" t="n">
         <v>20</v>
@@ -961,14 +961,14 @@
       <c r="F8" s="9" t="n">
         <v>46023</v>
       </c>
-      <c r="G8" s="3" t="s">
-        <v>11</v>
+      <c r="G8" s="1" t="s">
+        <v>13</v>
       </c>
       <c r="H8" s="11" t="n">
         <v>44197</v>
       </c>
       <c r="I8" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -976,7 +976,7 @@
         <v>103</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C9" s="1" t="n">
         <v>21</v>
@@ -990,8 +990,8 @@
       <c r="F9" s="9" t="n">
         <v>46023</v>
       </c>
-      <c r="G9" s="3" t="s">
-        <v>11</v>
+      <c r="G9" s="1" t="s">
+        <v>13</v>
       </c>
       <c r="H9" s="11" t="n">
         <v>44197</v>
@@ -1002,7 +1002,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="7" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C10" s="1" t="n">
         <v>22</v>
@@ -1016,14 +1016,14 @@
       <c r="F10" s="9" t="n">
         <v>46023</v>
       </c>
-      <c r="G10" s="3" t="s">
-        <v>11</v>
+      <c r="G10" s="1" t="s">
+        <v>13</v>
       </c>
       <c r="H10" s="11" t="n">
         <v>44927</v>
       </c>
       <c r="I10" s="1" t="s">
-        <v>22</v>
+        <v>13</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1037,7 +1037,7 @@
         <v>24</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E11" s="10" t="n">
         <v>0.12</v>
@@ -1045,8 +1045,8 @@
       <c r="F11" s="9" t="n">
         <v>46023</v>
       </c>
-      <c r="G11" s="3" t="s">
-        <v>11</v>
+      <c r="G11" s="1" t="s">
+        <v>13</v>
       </c>
       <c r="H11" s="9" t="n">
         <v>44562</v>
@@ -1066,7 +1066,7 @@
         <v>24</v>
       </c>
       <c r="D12" s="8" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E12" s="10" t="n">
         <v>0.12</v>
@@ -1074,8 +1074,8 @@
       <c r="F12" s="9" t="n">
         <v>46023</v>
       </c>
-      <c r="G12" s="3" t="s">
-        <v>11</v>
+      <c r="G12" s="1" t="s">
+        <v>13</v>
       </c>
       <c r="H12" s="9" t="n">
         <v>44562</v>
@@ -1092,7 +1092,7 @@
         <v>12</v>
       </c>
       <c r="D13" s="8" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E13" s="10" t="n">
         <v>0.088</v>
@@ -1100,14 +1100,14 @@
       <c r="F13" s="9" t="n">
         <v>46023</v>
       </c>
-      <c r="G13" s="3" t="s">
-        <v>11</v>
+      <c r="G13" s="1" t="s">
+        <v>13</v>
       </c>
       <c r="H13" s="9" t="n">
         <v>43831</v>
       </c>
       <c r="I13" s="1" t="s">
-        <v>22</v>
+        <v>13</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1118,7 +1118,7 @@
         <v>14</v>
       </c>
       <c r="D14" s="8" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E14" s="10" t="n">
         <v>0.088</v>
@@ -1126,14 +1126,14 @@
       <c r="F14" s="9" t="n">
         <v>46023</v>
       </c>
-      <c r="G14" s="3" t="s">
-        <v>11</v>
+      <c r="G14" s="1" t="s">
+        <v>13</v>
       </c>
       <c r="H14" s="9" t="n">
         <v>43831</v>
       </c>
       <c r="I14" s="1" t="s">
-        <v>22</v>
+        <v>13</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1152,11 +1152,11 @@
       <c r="F15" s="9" t="n">
         <v>45658</v>
       </c>
-      <c r="G15" s="3" t="s">
-        <v>11</v>
+      <c r="G15" s="1" t="s">
+        <v>13</v>
       </c>
       <c r="I15" s="1" t="s">
-        <v>22</v>
+        <v>13</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1175,11 +1175,11 @@
       <c r="F16" s="6" t="n">
         <v>45292</v>
       </c>
-      <c r="G16" s="3" t="s">
-        <v>11</v>
+      <c r="G16" s="1" t="s">
+        <v>13</v>
       </c>
       <c r="I16" s="1" t="s">
-        <v>22</v>
+        <v>13</v>
       </c>
     </row>
   </sheetData>

</xml_diff>